<commit_message>
[ADD] v19 Addons - 2
</commit_message>
<xml_diff>
--- a/script_migration_stock_config/static/data/Inventory Adj (stock.location).xlsx
+++ b/script_migration_stock_config/static/data/Inventory Adj (stock.location).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10917"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/waiyan/Project/Odoo/ppg/ppg/ppg/ppg/script_migration_stock_config/static/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9674026-7384-8740-A24F-84FC5AD2A52D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EE36D66-CDDC-864B-9FC6-4E8092156803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="80" yWindow="660" windowWidth="30160" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="203">
   <si>
     <t>Location Name</t>
   </si>
@@ -1054,7 +1054,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C193"/>
+  <dimension ref="A1:C191"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="46.83203125" customWidth="1"/>
@@ -1221,61 +1221,61 @@
         <v>120</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>117</v>
       </c>
       <c r="B16" t="s">
-        <v>74</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>117</v>
       </c>
       <c r="B17" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>69</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>117</v>
       </c>
       <c r="B18" t="s">
-        <v>69</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>189</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B19" t="s">
-        <v>82</v>
+        <v>15</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B20" t="s">
-        <v>70</v>
+        <v>16</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>189</v>
@@ -1283,10 +1283,10 @@
     </row>
     <row r="22" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B22" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>189</v>
@@ -1294,276 +1294,276 @@
     </row>
     <row r="23" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B23" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B24" t="s">
-        <v>18</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>189</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B25" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>126</v>
+        <v>197</v>
       </c>
       <c r="B26" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B27" t="s">
-        <v>20</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>197</v>
+        <v>129</v>
       </c>
       <c r="B28" t="s">
-        <v>60</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>189</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B29" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B30" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B31" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>131</v>
+        <v>191</v>
       </c>
       <c r="B32" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B33" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>191</v>
+        <v>134</v>
       </c>
       <c r="B34" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B35" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B36" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B37" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B38" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B39" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B40" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B41" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B42" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>141</v>
+        <v>198</v>
       </c>
       <c r="B43" t="s">
-        <v>34</v>
+        <v>92</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B44" t="s">
-        <v>35</v>
+        <v>94</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>198</v>
+        <v>144</v>
       </c>
       <c r="B45" t="s">
-        <v>92</v>
+        <v>36</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B46" t="s">
-        <v>94</v>
+        <v>37</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B47" t="s">
-        <v>36</v>
+        <v>93</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B48" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B49" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B50" t="s">
-        <v>38</v>
+        <v>40</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B51" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B52" t="s">
-        <v>40</v>
+        <v>66</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B53" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B54" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>189</v>
@@ -1571,10 +1571,10 @@
     </row>
     <row r="55" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B55" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>189</v>
@@ -1582,10 +1582,10 @@
     </row>
     <row r="56" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B56" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>189</v>
@@ -1593,32 +1593,29 @@
     </row>
     <row r="57" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B57" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B58" t="s">
-        <v>45</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>189</v>
+        <v>47</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B59" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>189</v>
@@ -1626,18 +1623,18 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B60" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B61" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>189</v>
@@ -1645,53 +1642,53 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B62" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B63" t="s">
-        <v>53</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>160</v>
-      </c>
-      <c r="B64" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B65" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>162</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>193</v>
+        <v>164</v>
+      </c>
+      <c r="B66" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B67" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>189</v>
@@ -1699,45 +1696,48 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B68" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B69" t="s">
-        <v>65</v>
-      </c>
-      <c r="C69" s="6" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B70" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B71" t="s">
-        <v>67</v>
+        <v>96</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B72" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C72" s="3" t="s">
         <v>189</v>
@@ -1745,10 +1745,10 @@
     </row>
     <row r="73" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B73" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C73" s="3" t="s">
         <v>189</v>
@@ -1756,10 +1756,10 @@
     </row>
     <row r="74" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>170</v>
-      </c>
-      <c r="B74" t="s">
-        <v>97</v>
+        <v>200</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>199</v>
       </c>
       <c r="C74" s="3" t="s">
         <v>189</v>
@@ -1767,10 +1767,10 @@
     </row>
     <row r="75" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>171</v>
+        <v>126</v>
       </c>
       <c r="B75" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C75" s="3" t="s">
         <v>189</v>
@@ -1778,10 +1778,10 @@
     </row>
     <row r="76" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>200</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>199</v>
+        <v>172</v>
+      </c>
+      <c r="B76" t="s">
+        <v>102</v>
       </c>
       <c r="C76" s="3" t="s">
         <v>189</v>
@@ -1789,10 +1789,10 @@
     </row>
     <row r="77" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>126</v>
+        <v>173</v>
       </c>
       <c r="B77" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C77" s="3" t="s">
         <v>189</v>
@@ -1800,10 +1800,10 @@
     </row>
     <row r="78" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B78" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C78" s="3" t="s">
         <v>189</v>
@@ -1811,10 +1811,10 @@
     </row>
     <row r="79" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>173</v>
+        <v>190</v>
       </c>
       <c r="B79" t="s">
-        <v>95</v>
+        <v>4</v>
       </c>
       <c r="C79" s="3" t="s">
         <v>189</v>
@@ -1822,10 +1822,10 @@
     </row>
     <row r="80" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B80" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C80" s="3" t="s">
         <v>189</v>
@@ -1833,10 +1833,10 @@
     </row>
     <row r="81" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>190</v>
+        <v>176</v>
       </c>
       <c r="B81" t="s">
-        <v>4</v>
+        <v>104</v>
       </c>
       <c r="C81" s="3" t="s">
         <v>189</v>
@@ -1844,10 +1844,10 @@
     </row>
     <row r="82" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B82" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C82" s="3" t="s">
         <v>189</v>
@@ -1855,10 +1855,10 @@
     </row>
     <row r="83" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B83" t="s">
-        <v>104</v>
+        <v>55</v>
       </c>
       <c r="C83" s="3" t="s">
         <v>189</v>
@@ -1866,10 +1866,10 @@
     </row>
     <row r="84" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B84" t="s">
-        <v>105</v>
+        <v>63</v>
       </c>
       <c r="C84" s="3" t="s">
         <v>189</v>
@@ -1877,10 +1877,10 @@
     </row>
     <row r="85" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B85" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C85" s="3" t="s">
         <v>189</v>
@@ -1888,10 +1888,10 @@
     </row>
     <row r="86" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>179</v>
-      </c>
-      <c r="B86" t="s">
-        <v>63</v>
+        <v>202</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>201</v>
       </c>
       <c r="C86" s="3" t="s">
         <v>189</v>
@@ -1899,10 +1899,10 @@
     </row>
     <row r="87" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B87" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C87" s="3" t="s">
         <v>189</v>
@@ -1910,10 +1910,10 @@
     </row>
     <row r="88" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>202</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>201</v>
+        <v>182</v>
+      </c>
+      <c r="B88" t="s">
+        <v>49</v>
       </c>
       <c r="C88" s="3" t="s">
         <v>189</v>
@@ -1921,10 +1921,10 @@
     </row>
     <row r="89" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B89" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="C89" s="3" t="s">
         <v>189</v>
@@ -1932,10 +1932,10 @@
     </row>
     <row r="90" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B90" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C90" s="3" t="s">
         <v>189</v>
@@ -1943,10 +1943,10 @@
     </row>
     <row r="91" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B91" t="s">
-        <v>48</v>
+        <v>106</v>
       </c>
       <c r="C91" s="3" t="s">
         <v>189</v>
@@ -1954,10 +1954,10 @@
     </row>
     <row r="92" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B92" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C92" s="3" t="s">
         <v>189</v>
@@ -1965,35 +1965,35 @@
     </row>
     <row r="93" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B93" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C93" s="3" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="94" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>186</v>
+        <v>117</v>
       </c>
       <c r="B94" t="s">
-        <v>21</v>
-      </c>
-      <c r="C94" s="3" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>77</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>187</v>
+        <v>117</v>
       </c>
       <c r="B95" t="s">
-        <v>107</v>
-      </c>
-      <c r="C95" s="3" t="s">
-        <v>189</v>
+        <v>71</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
@@ -2001,7 +2001,7 @@
         <v>117</v>
       </c>
       <c r="B96" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C96" s="4" t="s">
         <v>188</v>
@@ -2012,7 +2012,7 @@
         <v>117</v>
       </c>
       <c r="B97" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C97" s="4" t="s">
         <v>188</v>
@@ -2023,7 +2023,7 @@
         <v>117</v>
       </c>
       <c r="B98" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C98" s="4" t="s">
         <v>188</v>
@@ -2034,7 +2034,7 @@
         <v>117</v>
       </c>
       <c r="B99" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C99" s="4" t="s">
         <v>188</v>
@@ -2044,8 +2044,8 @@
       <c r="A100" t="s">
         <v>117</v>
       </c>
-      <c r="B100" t="s">
-        <v>75</v>
+      <c r="B100" s="5" t="s">
+        <v>192</v>
       </c>
       <c r="C100" s="4" t="s">
         <v>188</v>
@@ -2056,7 +2056,7 @@
         <v>117</v>
       </c>
       <c r="B101" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="C101" s="4" t="s">
         <v>188</v>
@@ -2066,8 +2066,8 @@
       <c r="A102" t="s">
         <v>117</v>
       </c>
-      <c r="B102" s="5" t="s">
-        <v>192</v>
+      <c r="B102" t="s">
+        <v>79</v>
       </c>
       <c r="C102" s="4" t="s">
         <v>188</v>
@@ -2078,7 +2078,7 @@
         <v>117</v>
       </c>
       <c r="B103" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C103" s="4" t="s">
         <v>188</v>
@@ -2089,29 +2089,29 @@
         <v>117</v>
       </c>
       <c r="B104" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C104" s="4" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A105" t="s">
-        <v>117</v>
-      </c>
-      <c r="B105" t="s">
-        <v>80</v>
+      <c r="A105" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B105" s="5" t="s">
+        <v>88</v>
       </c>
       <c r="C105" s="4" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A106" t="s">
-        <v>117</v>
-      </c>
-      <c r="B106" t="s">
-        <v>81</v>
+      <c r="A106" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B106" s="5" t="s">
+        <v>89</v>
       </c>
       <c r="C106" s="4" t="s">
         <v>188</v>
@@ -2122,7 +2122,7 @@
         <v>117</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C107" s="4" t="s">
         <v>188</v>
@@ -2133,7 +2133,7 @@
         <v>117</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C108" s="4" t="s">
         <v>188</v>
@@ -2144,7 +2144,7 @@
         <v>117</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C109" s="4" t="s">
         <v>188</v>
@@ -2155,7 +2155,7 @@
         <v>117</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C110" s="4" t="s">
         <v>188</v>
@@ -2166,32 +2166,32 @@
         <v>117</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C111" s="4" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A112" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="B112" s="5" t="s">
-        <v>82</v>
+    <row r="112" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A112" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="C112" s="4" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A113" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="B113" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C113" s="4" t="s">
-        <v>188</v>
+    <row r="113" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A113" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C113" s="3" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="114" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2210,41 +2210,29 @@
         <v>117</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="C115" s="3" t="s">
-        <v>189</v>
+        <v>195</v>
+      </c>
+      <c r="C115" s="4" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="116" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A116" s="2" t="s">
-        <v>117</v>
+        <v>162</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C116" s="4" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A117" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B117" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C117" s="4" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A118" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="B118" s="2" t="s">
         <v>196</v>
       </c>
+      <c r="C116" s="2"/>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A117" s="2"/>
+      <c r="B117" s="2"/>
+      <c r="C117" s="2"/>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A118" s="2"/>
+      <c r="B118" s="2"/>
       <c r="C118" s="2"/>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.2">
@@ -2612,27 +2600,17 @@
       <c r="B191" s="2"/>
       <c r="C191" s="2"/>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A192" s="2"/>
-      <c r="B192" s="2"/>
-      <c r="C192" s="2"/>
-    </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A193" s="2"/>
-      <c r="B193" s="2"/>
-      <c r="C193" s="2"/>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:A113 A115:A1048576">
+  <conditionalFormatting sqref="A113:A1048576 A1:A111">
     <cfRule type="duplicateValues" dxfId="3" priority="10"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A114">
+  <conditionalFormatting sqref="A112">
     <cfRule type="duplicateValues" dxfId="2" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B1:B113 B115:B1048576">
+  <conditionalFormatting sqref="B113:B1048576 B1:B111">
     <cfRule type="duplicateValues" dxfId="1" priority="12"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B114">
+  <conditionalFormatting sqref="B112">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>